<commit_message>
Added the AVCDL threat candidate ranking template (SP 800-30) workbook / updated the Threat Prioritization Plan - Candidate Ranking Procedure tertiary document (additional SP 800-30 material)
</commit_message>
<xml_diff>
--- a/source/reference_documents/templates/AVCDL threat candidate ranking template.xlsx
+++ b/source/reference_documents/templates/AVCDL threat candidate ranking template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9077B761-837A-ED45-97CC-C4717FB963BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C1EED1-3167-3F49-BF7B-E18C95A53F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-59900" yWindow="-31880" windowWidth="37960" windowHeight="22360" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
+    <workbookView xWindow="-59940" yWindow="-31880" windowWidth="37960" windowHeight="22360" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="7" r:id="rId1"/>
@@ -460,9 +460,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -493,7 +490,6 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -546,29 +542,33 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -911,18 +911,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="59" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="6"/>
@@ -937,19 +937,19 @@
       <c r="K3" s="6"/>
     </row>
     <row r="4" spans="2:11" ht="30" x14ac:dyDescent="0.3">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="51"/>
-      <c r="D4" s="52" t="s">
+      <c r="C4" s="48"/>
+      <c r="D4" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
       <c r="K4" s="6"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
@@ -965,19 +965,19 @@
       <c r="K5" s="6"/>
     </row>
     <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.3">
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="51"/>
-      <c r="D6" s="52" t="s">
+      <c r="C6" s="48"/>
+      <c r="D6" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="52"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
       <c r="K6" s="6"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
@@ -993,19 +993,19 @@
       <c r="K7" s="6"/>
     </row>
     <row r="8" spans="2:11" ht="30" x14ac:dyDescent="0.3">
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="53">
+      <c r="C8" s="48"/>
+      <c r="D8" s="55">
         <v>36765</v>
       </c>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -1021,11 +1021,11 @@
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="2:11" ht="30" x14ac:dyDescent="0.3">
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="51"/>
-      <c r="D10" s="54">
+      <c r="C10" s="48"/>
+      <c r="D10" s="49">
         <v>1</v>
       </c>
       <c r="E10" s="6"/>
@@ -1037,9 +1037,9 @@
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="2:11" ht="134" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -1049,18 +1049,18 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:11" ht="23" x14ac:dyDescent="0.2">
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
+      <c r="C12" s="53"/>
+      <c r="D12" s="53"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="53"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="53"/>
+      <c r="I12" s="53"/>
+      <c r="J12" s="53"/>
+      <c r="K12" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1090,11 +1090,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1106,99 +1106,99 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="44" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="47">
+      <c r="B5" s="45">
         <v>1</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="48" t="s">
+      <c r="C5" s="42"/>
+      <c r="D5" s="46" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="47"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="48"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="46"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="47"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="48"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="46"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="47"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="48"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="46"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="47"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="48"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="46"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="47"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="48"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="46"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="47"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="48"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="46"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="47"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="48"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="46"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="47"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="48"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="46"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="47"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="48"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="46"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="47"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="48"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="46"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="47"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="48"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="46"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="47"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="48"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="46"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="47"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="48"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="46"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="47"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="48"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="46"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="47"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="48"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1219,11 +1219,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1235,10 +1235,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="38" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -1246,96 +1246,96 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="17" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="43"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="35"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="33"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="43"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="35"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="33"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="43"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="35"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="33"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="43"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="35"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="33"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="43"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="35"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="33"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="43"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="35"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="43"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="35"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="33"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="43"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="35"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="33"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="35"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="33"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="43"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="35"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="33"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="43"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="35"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="33"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="43"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="35"/>
+      <c r="B18" s="41"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="33"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="43"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="35"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="43"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="35"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1362,17 +1362,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1390,28 +1390,28 @@
     </row>
     <row r="4" spans="1:13" ht="49" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="11" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="24" t="s">
         <v>23</v>
       </c>
       <c r="J4" s="4" t="s">
@@ -1419,276 +1419,276 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="24" t="str">
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="23" t="str">
         <f>VLOOKUP(G5,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I5" s="24" t="str">
+      <c r="I5" s="23" t="str">
         <f>VLOOKUP(G5,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J5" s="19"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="24" t="str">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="23" t="str">
         <f>VLOOKUP(G6,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I6" s="24" t="str">
+      <c r="I6" s="23" t="str">
         <f>VLOOKUP(G6,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J6" s="19"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="24" t="str">
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="23" t="str">
         <f>VLOOKUP(G7,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I7" s="24" t="str">
+      <c r="I7" s="23" t="str">
         <f>VLOOKUP(G7,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J7" s="23"/>
+      <c r="J7" s="22"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="24" t="str">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="23" t="str">
         <f>VLOOKUP(G8,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I8" s="24" t="str">
+      <c r="I8" s="23" t="str">
         <f>VLOOKUP(G8,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J8" s="23"/>
+      <c r="J8" s="22"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="24" t="str">
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="23" t="str">
         <f>VLOOKUP(G9,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I9" s="24" t="str">
+      <c r="I9" s="23" t="str">
         <f>VLOOKUP(G9,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J9" s="23"/>
+      <c r="J9" s="22"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="24" t="str">
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="23" t="str">
         <f>VLOOKUP(G10,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I10" s="24" t="str">
+      <c r="I10" s="23" t="str">
         <f>VLOOKUP(G10,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J10" s="23"/>
+      <c r="J10" s="22"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="24" t="str">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="23" t="str">
         <f>VLOOKUP(G11,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I11" s="24" t="str">
+      <c r="I11" s="23" t="str">
         <f>VLOOKUP(G11,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J11" s="23"/>
+      <c r="J11" s="22"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="24" t="str">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="23" t="str">
         <f>VLOOKUP(G12,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I12" s="24" t="str">
+      <c r="I12" s="23" t="str">
         <f>VLOOKUP(G12,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J12" s="23"/>
+      <c r="J12" s="22"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="24" t="str">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="23" t="str">
         <f>VLOOKUP(G13,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I13" s="24" t="str">
+      <c r="I13" s="23" t="str">
         <f>VLOOKUP(G13,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J13" s="23"/>
+      <c r="J13" s="22"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="24" t="str">
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="23" t="str">
         <f>VLOOKUP(G14,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I14" s="24" t="str">
+      <c r="I14" s="23" t="str">
         <f>VLOOKUP(G14,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J14" s="23"/>
+      <c r="J14" s="22"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="24" t="str">
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="23" t="str">
         <f>VLOOKUP(G15,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I15" s="24" t="str">
+      <c r="I15" s="23" t="str">
         <f>VLOOKUP(G15,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J15" s="23"/>
+      <c r="J15" s="22"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="24" t="str">
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="23" t="str">
         <f>VLOOKUP(G16,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I16" s="24" t="str">
+      <c r="I16" s="23" t="str">
         <f>VLOOKUP(G16,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J16" s="23"/>
+      <c r="J16" s="22"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="24" t="str">
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="23" t="str">
         <f>VLOOKUP(G17,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I17" s="24" t="str">
+      <c r="I17" s="23" t="str">
         <f>VLOOKUP(G17,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J17" s="23"/>
+      <c r="J17" s="22"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="24" t="str">
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="23" t="str">
         <f>VLOOKUP(G18,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I18" s="24" t="str">
+      <c r="I18" s="23" t="str">
         <f>VLOOKUP(G18,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J18" s="23"/>
+      <c r="J18" s="22"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="24" t="str">
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="23" t="str">
         <f>VLOOKUP(G19,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I19" s="24" t="str">
+      <c r="I19" s="23" t="str">
         <f>VLOOKUP(G19,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J19" s="23"/>
+      <c r="J19" s="22"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="24" t="str">
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="23" t="str">
         <f>VLOOKUP(G20,[0]!RQ_start:RQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="I20" s="24" t="str">
+      <c r="I20" s="23" t="str">
         <f>VLOOKUP(G20,[0]!DQ_start:DQ_end,2,TRUE)</f>
         <v>none</v>
       </c>
-      <c r="J20" s="23"/>
+      <c r="J20" s="22"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B21" s="6"/>
@@ -1779,17 +1779,17 @@
       <c r="J28" s="6"/>
     </row>
     <row r="29" spans="2:10" ht="20" x14ac:dyDescent="0.2">
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="57"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
@@ -1966,12 +1966,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -1984,10 +1984,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -1998,110 +1998,110 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="27">
+      <c r="B5" s="25">
         <v>0</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="27" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B6" s="27">
+      <c r="B6" s="25">
         <v>1E-4</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="32"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="33"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="32"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B8" s="33"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="32"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B9" s="33"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="30"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B10" s="34"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="14"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="13"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B11" s="34"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="13"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B12" s="34"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="14"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B14" s="34"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B15" s="34"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B16" s="34"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="34"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="38"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="36"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19" s="33"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="30"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B20" s="33"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="32"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="30"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -2123,12 +2123,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -2141,10 +2141,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -2155,110 +2155,110 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="27">
+      <c r="B5" s="25">
         <v>0</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="27" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B6" s="27">
+      <c r="B6" s="25">
         <v>1E-4</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="32"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="33"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="32"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B8" s="33"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="32"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B9" s="33"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="30"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B10" s="34"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="14"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="13"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B11" s="34"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="14"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="13"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B12" s="34"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="14"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B13" s="34"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B14" s="34"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B15" s="34"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B16" s="34"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="34"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="38"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="36"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19" s="33"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="30"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B20" s="33"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="32"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="30"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -2291,18 +2291,18 @@
       <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="56"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
+      <c r="A2" s="50"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="56"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="57"/>
+      <c r="A3" s="50"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="51"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="7"/>
-      <c r="B4" s="57"/>
+      <c r="B4" s="51"/>
       <c r="C4" s="7"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>